<commit_message>
chore(ci): add lint script and complete full pipeline verification
</commit_message>
<xml_diff>
--- a/FINAL REPORTS/Vulnerability_Test_Report.xlsx
+++ b/FINAL REPORTS/Vulnerability_Test_Report.xlsx
@@ -53,7 +53,7 @@
     <t>TOTAL SCAN DURATION</t>
   </si>
   <si>
-    <t>0.13s</t>
+    <t>0.12s</t>
   </si>
   <si>
     <t>Automated DAST Runner Node</t>
@@ -62,7 +62,7 @@
     <t>ASSESSMENT TIMESTAMP</t>
   </si>
   <si>
-    <t>6/8/2026, 7:11:33 pm</t>
+    <t>7/8/2026, 11:05:23 am</t>
   </si>
   <si>
     <t>CI/CD Pipeline Security Gate</t>
@@ -3247,7 +3247,7 @@
         <v>67</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -3282,7 +3282,7 @@
         <v>67</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -3317,7 +3317,7 @@
         <v>67</v>
       </c>
       <c r="K4">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -3352,7 +3352,7 @@
         <v>67</v>
       </c>
       <c r="K5">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3387,7 +3387,7 @@
         <v>67</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -3457,7 +3457,7 @@
         <v>67</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -3492,7 +3492,7 @@
         <v>67</v>
       </c>
       <c r="K9">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -3527,7 +3527,7 @@
         <v>67</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -3562,7 +3562,7 @@
         <v>67</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -3597,7 +3597,7 @@
         <v>67</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -3632,7 +3632,7 @@
         <v>67</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3667,7 +3667,7 @@
         <v>67</v>
       </c>
       <c r="K14">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -3702,7 +3702,7 @@
         <v>67</v>
       </c>
       <c r="K15">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -3737,7 +3737,7 @@
         <v>67</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>67</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3807,7 +3807,7 @@
         <v>67</v>
       </c>
       <c r="K18">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -3842,7 +3842,7 @@
         <v>67</v>
       </c>
       <c r="K19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -3877,7 +3877,7 @@
         <v>67</v>
       </c>
       <c r="K20">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -3912,7 +3912,7 @@
         <v>67</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -3947,7 +3947,7 @@
         <v>67</v>
       </c>
       <c r="K22">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -3982,7 +3982,7 @@
         <v>67</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -4017,7 +4017,7 @@
         <v>67</v>
       </c>
       <c r="K24">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -4052,7 +4052,7 @@
         <v>67</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -4087,7 +4087,7 @@
         <v>67</v>
       </c>
       <c r="K26">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -4122,7 +4122,7 @@
         <v>67</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -4192,7 +4192,7 @@
         <v>67</v>
       </c>
       <c r="K29">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -4227,7 +4227,7 @@
         <v>67</v>
       </c>
       <c r="K30">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -4297,7 +4297,7 @@
         <v>67</v>
       </c>
       <c r="K32">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -4332,7 +4332,7 @@
         <v>67</v>
       </c>
       <c r="K33">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -4367,7 +4367,7 @@
         <v>67</v>
       </c>
       <c r="K34">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -4402,7 +4402,7 @@
         <v>67</v>
       </c>
       <c r="K35">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -4472,7 +4472,7 @@
         <v>67</v>
       </c>
       <c r="K37">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -4507,7 +4507,7 @@
         <v>67</v>
       </c>
       <c r="K38">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -4542,7 +4542,7 @@
         <v>67</v>
       </c>
       <c r="K39">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -4577,7 +4577,7 @@
         <v>67</v>
       </c>
       <c r="K40">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -4612,7 +4612,7 @@
         <v>67</v>
       </c>
       <c r="K41">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -4647,7 +4647,7 @@
         <v>67</v>
       </c>
       <c r="K42">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -4682,7 +4682,7 @@
         <v>67</v>
       </c>
       <c r="K43">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -4717,7 +4717,7 @@
         <v>67</v>
       </c>
       <c r="K44">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -4787,7 +4787,7 @@
         <v>67</v>
       </c>
       <c r="K46">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -4822,7 +4822,7 @@
         <v>67</v>
       </c>
       <c r="K47">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -4857,7 +4857,7 @@
         <v>67</v>
       </c>
       <c r="K48">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -4892,7 +4892,7 @@
         <v>67</v>
       </c>
       <c r="K49">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -4927,7 +4927,7 @@
         <v>67</v>
       </c>
       <c r="K50">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -4997,7 +4997,7 @@
         <v>67</v>
       </c>
       <c r="K52">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -5032,7 +5032,7 @@
         <v>67</v>
       </c>
       <c r="K53">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -5067,7 +5067,7 @@
         <v>67</v>
       </c>
       <c r="K54">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -5102,7 +5102,7 @@
         <v>67</v>
       </c>
       <c r="K55">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -5137,7 +5137,7 @@
         <v>67</v>
       </c>
       <c r="K56">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -5172,7 +5172,7 @@
         <v>67</v>
       </c>
       <c r="K57">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
@@ -5207,7 +5207,7 @@
         <v>67</v>
       </c>
       <c r="K58">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -5242,7 +5242,7 @@
         <v>67</v>
       </c>
       <c r="K59">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
@@ -5277,7 +5277,7 @@
         <v>67</v>
       </c>
       <c r="K60">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -5312,7 +5312,7 @@
         <v>67</v>
       </c>
       <c r="K61">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -5347,7 +5347,7 @@
         <v>67</v>
       </c>
       <c r="K62">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -5382,7 +5382,7 @@
         <v>67</v>
       </c>
       <c r="K63">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -5417,7 +5417,7 @@
         <v>67</v>
       </c>
       <c r="K64">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -5452,7 +5452,7 @@
         <v>67</v>
       </c>
       <c r="K65">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -5487,7 +5487,7 @@
         <v>67</v>
       </c>
       <c r="K66">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -5522,7 +5522,7 @@
         <v>67</v>
       </c>
       <c r="K67">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -5557,7 +5557,7 @@
         <v>67</v>
       </c>
       <c r="K68">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -5627,7 +5627,7 @@
         <v>67</v>
       </c>
       <c r="K70">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -5732,7 +5732,7 @@
         <v>67</v>
       </c>
       <c r="K73">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -5767,7 +5767,7 @@
         <v>67</v>
       </c>
       <c r="K74">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -5802,7 +5802,7 @@
         <v>67</v>
       </c>
       <c r="K75">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -5872,7 +5872,7 @@
         <v>67</v>
       </c>
       <c r="K77">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -5907,7 +5907,7 @@
         <v>67</v>
       </c>
       <c r="K78">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
@@ -5942,7 +5942,7 @@
         <v>67</v>
       </c>
       <c r="K79">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -5977,7 +5977,7 @@
         <v>67</v>
       </c>
       <c r="K80">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -6012,7 +6012,7 @@
         <v>67</v>
       </c>
       <c r="K81">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -6047,7 +6047,7 @@
         <v>67</v>
       </c>
       <c r="K82">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -6082,7 +6082,7 @@
         <v>67</v>
       </c>
       <c r="K83">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -6117,7 +6117,7 @@
         <v>67</v>
       </c>
       <c r="K84">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -6152,7 +6152,7 @@
         <v>67</v>
       </c>
       <c r="K85">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -6187,7 +6187,7 @@
         <v>67</v>
       </c>
       <c r="K86">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -6222,7 +6222,7 @@
         <v>67</v>
       </c>
       <c r="K87">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
@@ -6257,7 +6257,7 @@
         <v>67</v>
       </c>
       <c r="K88">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -6292,7 +6292,7 @@
         <v>67</v>
       </c>
       <c r="K89">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
@@ -6327,7 +6327,7 @@
         <v>67</v>
       </c>
       <c r="K90">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
@@ -6362,7 +6362,7 @@
         <v>67</v>
       </c>
       <c r="K91">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
@@ -6397,7 +6397,7 @@
         <v>67</v>
       </c>
       <c r="K92">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
@@ -6432,7 +6432,7 @@
         <v>67</v>
       </c>
       <c r="K93">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -6467,7 +6467,7 @@
         <v>67</v>
       </c>
       <c r="K94">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
@@ -6502,7 +6502,7 @@
         <v>67</v>
       </c>
       <c r="K95">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
@@ -6537,7 +6537,7 @@
         <v>67</v>
       </c>
       <c r="K96">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
@@ -6572,7 +6572,7 @@
         <v>67</v>
       </c>
       <c r="K97">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
@@ -6607,7 +6607,7 @@
         <v>67</v>
       </c>
       <c r="K98">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -6642,7 +6642,7 @@
         <v>67</v>
       </c>
       <c r="K99">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -6677,7 +6677,7 @@
         <v>67</v>
       </c>
       <c r="K100">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
@@ -6712,7 +6712,7 @@
         <v>67</v>
       </c>
       <c r="K101">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -6817,7 +6817,7 @@
         <v>67</v>
       </c>
       <c r="K104">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -6852,7 +6852,7 @@
         <v>67</v>
       </c>
       <c r="K105">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
@@ -6887,7 +6887,7 @@
         <v>67</v>
       </c>
       <c r="K106">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
@@ -6922,7 +6922,7 @@
         <v>67</v>
       </c>
       <c r="K107">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -6957,7 +6957,7 @@
         <v>67</v>
       </c>
       <c r="K108">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
@@ -7027,7 +7027,7 @@
         <v>67</v>
       </c>
       <c r="K110">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
@@ -7062,7 +7062,7 @@
         <v>67</v>
       </c>
       <c r="K111">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
@@ -7097,7 +7097,7 @@
         <v>67</v>
       </c>
       <c r="K112">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
@@ -7167,7 +7167,7 @@
         <v>67</v>
       </c>
       <c r="K114">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
@@ -7202,7 +7202,7 @@
         <v>67</v>
       </c>
       <c r="K115">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
@@ -7237,7 +7237,7 @@
         <v>67</v>
       </c>
       <c r="K116">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
@@ -7272,7 +7272,7 @@
         <v>67</v>
       </c>
       <c r="K117">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
@@ -7307,7 +7307,7 @@
         <v>67</v>
       </c>
       <c r="K118">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
@@ -7342,7 +7342,7 @@
         <v>67</v>
       </c>
       <c r="K119">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
@@ -7377,7 +7377,7 @@
         <v>67</v>
       </c>
       <c r="K120">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
@@ -7412,7 +7412,7 @@
         <v>67</v>
       </c>
       <c r="K121">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
@@ -7447,7 +7447,7 @@
         <v>67</v>
       </c>
       <c r="K122">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -7482,7 +7482,7 @@
         <v>67</v>
       </c>
       <c r="K123">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
@@ -7517,7 +7517,7 @@
         <v>67</v>
       </c>
       <c r="K124">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
@@ -7552,7 +7552,7 @@
         <v>67</v>
       </c>
       <c r="K125">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -7587,7 +7587,7 @@
         <v>67</v>
       </c>
       <c r="K126">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
@@ -7657,7 +7657,7 @@
         <v>67</v>
       </c>
       <c r="K128">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
@@ -7692,7 +7692,7 @@
         <v>67</v>
       </c>
       <c r="K129">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
@@ -7727,7 +7727,7 @@
         <v>67</v>
       </c>
       <c r="K130">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.25">
@@ -7762,7 +7762,7 @@
         <v>67</v>
       </c>
       <c r="K131">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
@@ -7797,7 +7797,7 @@
         <v>67</v>
       </c>
       <c r="K132">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.25">
@@ -7832,7 +7832,7 @@
         <v>67</v>
       </c>
       <c r="K133">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.25">
@@ -7867,7 +7867,7 @@
         <v>67</v>
       </c>
       <c r="K134">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
@@ -7902,7 +7902,7 @@
         <v>67</v>
       </c>
       <c r="K135">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.25">
@@ -7937,7 +7937,7 @@
         <v>67</v>
       </c>
       <c r="K136">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
@@ -8007,7 +8007,7 @@
         <v>67</v>
       </c>
       <c r="K138">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.25">
@@ -8042,7 +8042,7 @@
         <v>67</v>
       </c>
       <c r="K139">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.25">
@@ -8077,7 +8077,7 @@
         <v>67</v>
       </c>
       <c r="K140">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.25">
@@ -8112,7 +8112,7 @@
         <v>67</v>
       </c>
       <c r="K141">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.25">
@@ -8217,7 +8217,7 @@
         <v>67</v>
       </c>
       <c r="K144">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.25">
@@ -8252,7 +8252,7 @@
         <v>67</v>
       </c>
       <c r="K145">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
@@ -8287,7 +8287,7 @@
         <v>67</v>
       </c>
       <c r="K146">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.25">
@@ -8322,7 +8322,7 @@
         <v>67</v>
       </c>
       <c r="K147">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.25">
@@ -8357,7 +8357,7 @@
         <v>67</v>
       </c>
       <c r="K148">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.25">
@@ -8427,7 +8427,7 @@
         <v>67</v>
       </c>
       <c r="K150">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
@@ -8462,7 +8462,7 @@
         <v>67</v>
       </c>
       <c r="K151">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
@@ -8497,7 +8497,7 @@
         <v>67</v>
       </c>
       <c r="K152">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
@@ -8532,7 +8532,7 @@
         <v>67</v>
       </c>
       <c r="K153">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
@@ -8567,7 +8567,7 @@
         <v>67</v>
       </c>
       <c r="K154">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
@@ -8602,7 +8602,7 @@
         <v>67</v>
       </c>
       <c r="K155">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
@@ -8637,7 +8637,7 @@
         <v>67</v>
       </c>
       <c r="K156">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
@@ -8672,7 +8672,7 @@
         <v>67</v>
       </c>
       <c r="K157">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
@@ -8707,7 +8707,7 @@
         <v>67</v>
       </c>
       <c r="K158">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
@@ -8777,7 +8777,7 @@
         <v>67</v>
       </c>
       <c r="K160">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.25">
@@ -8812,7 +8812,7 @@
         <v>67</v>
       </c>
       <c r="K161">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
@@ -8847,7 +8847,7 @@
         <v>67</v>
       </c>
       <c r="K162">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
@@ -8882,7 +8882,7 @@
         <v>67</v>
       </c>
       <c r="K163">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.25">
@@ -8917,7 +8917,7 @@
         <v>67</v>
       </c>
       <c r="K164">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.25">
@@ -8952,7 +8952,7 @@
         <v>67</v>
       </c>
       <c r="K165">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.25">
@@ -8987,7 +8987,7 @@
         <v>67</v>
       </c>
       <c r="K166">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.25">
@@ -9022,7 +9022,7 @@
         <v>67</v>
       </c>
       <c r="K167">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.25">
@@ -9057,7 +9057,7 @@
         <v>67</v>
       </c>
       <c r="K168">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.25">
@@ -9092,7 +9092,7 @@
         <v>67</v>
       </c>
       <c r="K169">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.25">
@@ -9127,7 +9127,7 @@
         <v>67</v>
       </c>
       <c r="K170">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.25">
@@ -9162,7 +9162,7 @@
         <v>67</v>
       </c>
       <c r="K171">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.25">
@@ -9197,7 +9197,7 @@
         <v>67</v>
       </c>
       <c r="K172">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
@@ -9232,7 +9232,7 @@
         <v>67</v>
       </c>
       <c r="K173">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
@@ -9267,7 +9267,7 @@
         <v>67</v>
       </c>
       <c r="K174">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
@@ -9302,7 +9302,7 @@
         <v>67</v>
       </c>
       <c r="K175">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.25">
@@ -9337,7 +9337,7 @@
         <v>67</v>
       </c>
       <c r="K176">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
@@ -9372,7 +9372,7 @@
         <v>67</v>
       </c>
       <c r="K177">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
@@ -9407,7 +9407,7 @@
         <v>67</v>
       </c>
       <c r="K178">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
@@ -9442,7 +9442,7 @@
         <v>67</v>
       </c>
       <c r="K179">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
@@ -9512,7 +9512,7 @@
         <v>67</v>
       </c>
       <c r="K181">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
@@ -9547,7 +9547,7 @@
         <v>67</v>
       </c>
       <c r="K182">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
@@ -9582,7 +9582,7 @@
         <v>67</v>
       </c>
       <c r="K183">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
@@ -9617,7 +9617,7 @@
         <v>67</v>
       </c>
       <c r="K184">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.25">
@@ -9652,7 +9652,7 @@
         <v>67</v>
       </c>
       <c r="K185">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.25">
@@ -9687,7 +9687,7 @@
         <v>67</v>
       </c>
       <c r="K186">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
@@ -9722,7 +9722,7 @@
         <v>67</v>
       </c>
       <c r="K187">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
@@ -9757,7 +9757,7 @@
         <v>67</v>
       </c>
       <c r="K188">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>67</v>
       </c>
       <c r="K191">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.25">
@@ -9932,7 +9932,7 @@
         <v>67</v>
       </c>
       <c r="K193">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.25">
@@ -9967,7 +9967,7 @@
         <v>67</v>
       </c>
       <c r="K194">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.25">
@@ -10002,7 +10002,7 @@
         <v>67</v>
       </c>
       <c r="K195">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.25">
@@ -10037,7 +10037,7 @@
         <v>67</v>
       </c>
       <c r="K196">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.25">
@@ -10072,7 +10072,7 @@
         <v>67</v>
       </c>
       <c r="K197">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198" spans="1:11" x14ac:dyDescent="0.25">
@@ -10107,7 +10107,7 @@
         <v>67</v>
       </c>
       <c r="K198">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="199" spans="1:11" x14ac:dyDescent="0.25">
@@ -10142,7 +10142,7 @@
         <v>67</v>
       </c>
       <c r="K199">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
@@ -10177,7 +10177,7 @@
         <v>67</v>
       </c>
       <c r="K200">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.25">
@@ -10212,7 +10212,7 @@
         <v>67</v>
       </c>
       <c r="K201">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.25">
@@ -10247,7 +10247,7 @@
         <v>67</v>
       </c>
       <c r="K202">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.25">
@@ -10282,7 +10282,7 @@
         <v>67</v>
       </c>
       <c r="K203">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.25">
@@ -10352,7 +10352,7 @@
         <v>67</v>
       </c>
       <c r="K205">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="206" spans="1:11" x14ac:dyDescent="0.25">
@@ -10387,7 +10387,7 @@
         <v>67</v>
       </c>
       <c r="K206">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.25">
@@ -10422,7 +10422,7 @@
         <v>67</v>
       </c>
       <c r="K207">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:11" x14ac:dyDescent="0.25">
@@ -10457,7 +10457,7 @@
         <v>67</v>
       </c>
       <c r="K208">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209" spans="1:11" x14ac:dyDescent="0.25">
@@ -10492,7 +10492,7 @@
         <v>67</v>
       </c>
       <c r="K209">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.25">
@@ -10527,7 +10527,7 @@
         <v>67</v>
       </c>
       <c r="K210">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.25">
@@ -10562,7 +10562,7 @@
         <v>67</v>
       </c>
       <c r="K211">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.25">
@@ -10632,7 +10632,7 @@
         <v>67</v>
       </c>
       <c r="K213">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
@@ -10667,7 +10667,7 @@
         <v>67</v>
       </c>
       <c r="K214">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
@@ -10702,7 +10702,7 @@
         <v>67</v>
       </c>
       <c r="K215">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216" spans="1:11" x14ac:dyDescent="0.25">
@@ -10737,7 +10737,7 @@
         <v>67</v>
       </c>
       <c r="K216">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="217" spans="1:11" x14ac:dyDescent="0.25">
@@ -10772,7 +10772,7 @@
         <v>67</v>
       </c>
       <c r="K217">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.25">
@@ -10807,7 +10807,7 @@
         <v>67</v>
       </c>
       <c r="K218">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.25">
@@ -10842,7 +10842,7 @@
         <v>67</v>
       </c>
       <c r="K219">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" spans="1:11" x14ac:dyDescent="0.25">
@@ -10877,7 +10877,7 @@
         <v>67</v>
       </c>
       <c r="K220">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
@@ -10912,7 +10912,7 @@
         <v>67</v>
       </c>
       <c r="K221">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
@@ -10947,7 +10947,7 @@
         <v>67</v>
       </c>
       <c r="K222">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
@@ -11017,7 +11017,7 @@
         <v>67</v>
       </c>
       <c r="K224">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="225" spans="1:11" x14ac:dyDescent="0.25">
@@ -11052,7 +11052,7 @@
         <v>67</v>
       </c>
       <c r="K225">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="226" spans="1:11" x14ac:dyDescent="0.25">
@@ -11087,7 +11087,7 @@
         <v>67</v>
       </c>
       <c r="K226">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227" spans="1:11" x14ac:dyDescent="0.25">
@@ -11122,7 +11122,7 @@
         <v>67</v>
       </c>
       <c r="K227">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228" spans="1:11" x14ac:dyDescent="0.25">
@@ -11157,7 +11157,7 @@
         <v>67</v>
       </c>
       <c r="K228">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229" spans="1:11" x14ac:dyDescent="0.25">
@@ -11192,7 +11192,7 @@
         <v>67</v>
       </c>
       <c r="K229">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="230" spans="1:11" x14ac:dyDescent="0.25">
@@ -11227,7 +11227,7 @@
         <v>67</v>
       </c>
       <c r="K230">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.25">
@@ -11262,7 +11262,7 @@
         <v>67</v>
       </c>
       <c r="K231">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="232" spans="1:11" x14ac:dyDescent="0.25">
@@ -11297,7 +11297,7 @@
         <v>67</v>
       </c>
       <c r="K232">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="233" spans="1:11" x14ac:dyDescent="0.25">
@@ -11332,7 +11332,7 @@
         <v>67</v>
       </c>
       <c r="K233">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="234" spans="1:11" x14ac:dyDescent="0.25">
@@ -11437,7 +11437,7 @@
         <v>67</v>
       </c>
       <c r="K236">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.25">
@@ -11507,7 +11507,7 @@
         <v>67</v>
       </c>
       <c r="K238">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="1:11" x14ac:dyDescent="0.25">
@@ -11577,7 +11577,7 @@
         <v>67</v>
       </c>
       <c r="K240">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -11647,7 +11647,7 @@
         <v>67</v>
       </c>
       <c r="K242">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
@@ -11682,7 +11682,7 @@
         <v>67</v>
       </c>
       <c r="K243">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
@@ -11717,7 +11717,7 @@
         <v>67</v>
       </c>
       <c r="K244">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
@@ -11752,7 +11752,7 @@
         <v>67</v>
       </c>
       <c r="K245">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="246" spans="1:11" x14ac:dyDescent="0.25">
@@ -11787,7 +11787,7 @@
         <v>67</v>
       </c>
       <c r="K246">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.25">
@@ -11822,7 +11822,7 @@
         <v>67</v>
       </c>
       <c r="K247">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="248" spans="1:11" x14ac:dyDescent="0.25">
@@ -11892,7 +11892,7 @@
         <v>67</v>
       </c>
       <c r="K249">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -11927,7 +11927,7 @@
         <v>67</v>
       </c>
       <c r="K250">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="251" spans="1:11" x14ac:dyDescent="0.25">
@@ -11962,7 +11962,7 @@
         <v>67</v>
       </c>
       <c r="K251">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.25">
@@ -11997,7 +11997,7 @@
         <v>67</v>
       </c>
       <c r="K252">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.25">
@@ -12032,7 +12032,7 @@
         <v>67</v>
       </c>
       <c r="K253">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.25">
@@ -12102,7 +12102,7 @@
         <v>67</v>
       </c>
       <c r="K255">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.25">
@@ -12137,7 +12137,7 @@
         <v>67</v>
       </c>
       <c r="K256">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="257" spans="1:11" x14ac:dyDescent="0.25">
@@ -12172,7 +12172,7 @@
         <v>67</v>
       </c>
       <c r="K257">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.25">
@@ -12207,7 +12207,7 @@
         <v>67</v>
       </c>
       <c r="K258">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="259" spans="1:11" x14ac:dyDescent="0.25">
@@ -12277,7 +12277,7 @@
         <v>67</v>
       </c>
       <c r="K260">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="261" spans="1:11" x14ac:dyDescent="0.25">
@@ -12312,7 +12312,7 @@
         <v>67</v>
       </c>
       <c r="K261">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="262" spans="1:11" x14ac:dyDescent="0.25">
@@ -12347,7 +12347,7 @@
         <v>67</v>
       </c>
       <c r="K262">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="263" spans="1:11" x14ac:dyDescent="0.25">
@@ -12382,7 +12382,7 @@
         <v>67</v>
       </c>
       <c r="K263">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="264" spans="1:11" x14ac:dyDescent="0.25">
@@ -12417,7 +12417,7 @@
         <v>67</v>
       </c>
       <c r="K264">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="265" spans="1:11" x14ac:dyDescent="0.25">
@@ -12452,7 +12452,7 @@
         <v>67</v>
       </c>
       <c r="K265">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="266" spans="1:11" x14ac:dyDescent="0.25">
@@ -12487,7 +12487,7 @@
         <v>67</v>
       </c>
       <c r="K266">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="267" spans="1:11" x14ac:dyDescent="0.25">
@@ -12522,7 +12522,7 @@
         <v>67</v>
       </c>
       <c r="K267">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="268" spans="1:11" x14ac:dyDescent="0.25">
@@ -12557,7 +12557,7 @@
         <v>67</v>
       </c>
       <c r="K268">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="269" spans="1:11" x14ac:dyDescent="0.25">
@@ -12592,7 +12592,7 @@
         <v>67</v>
       </c>
       <c r="K269">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="270" spans="1:11" x14ac:dyDescent="0.25">
@@ -12627,7 +12627,7 @@
         <v>67</v>
       </c>
       <c r="K270">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="271" spans="1:11" x14ac:dyDescent="0.25">
@@ -12662,7 +12662,7 @@
         <v>67</v>
       </c>
       <c r="K271">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="272" spans="1:11" x14ac:dyDescent="0.25">
@@ -12697,7 +12697,7 @@
         <v>67</v>
       </c>
       <c r="K272">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.25">
@@ -12732,7 +12732,7 @@
         <v>67</v>
       </c>
       <c r="K273">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="274" spans="1:11" x14ac:dyDescent="0.25">
@@ -12767,7 +12767,7 @@
         <v>67</v>
       </c>
       <c r="K274">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="275" spans="1:11" x14ac:dyDescent="0.25">
@@ -12837,7 +12837,7 @@
         <v>67</v>
       </c>
       <c r="K276">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="277" spans="1:11" x14ac:dyDescent="0.25">
@@ -12872,7 +12872,7 @@
         <v>67</v>
       </c>
       <c r="K277">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="278" spans="1:11" x14ac:dyDescent="0.25">
@@ -12907,7 +12907,7 @@
         <v>67</v>
       </c>
       <c r="K278">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="279" spans="1:11" x14ac:dyDescent="0.25">
@@ -12942,7 +12942,7 @@
         <v>67</v>
       </c>
       <c r="K279">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="280" spans="1:11" x14ac:dyDescent="0.25">
@@ -13012,7 +13012,7 @@
         <v>67</v>
       </c>
       <c r="K281">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="282" spans="1:11" x14ac:dyDescent="0.25">
@@ -13047,7 +13047,7 @@
         <v>67</v>
       </c>
       <c r="K282">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="283" spans="1:11" x14ac:dyDescent="0.25">
@@ -13117,7 +13117,7 @@
         <v>67</v>
       </c>
       <c r="K284">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="285" spans="1:11" x14ac:dyDescent="0.25">
@@ -13152,7 +13152,7 @@
         <v>67</v>
       </c>
       <c r="K285">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="286" spans="1:11" x14ac:dyDescent="0.25">
@@ -13222,7 +13222,7 @@
         <v>67</v>
       </c>
       <c r="K287">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="288" spans="1:11" x14ac:dyDescent="0.25">
@@ -13257,7 +13257,7 @@
         <v>67</v>
       </c>
       <c r="K288">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="289" spans="1:11" x14ac:dyDescent="0.25">
@@ -13292,7 +13292,7 @@
         <v>67</v>
       </c>
       <c r="K289">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="290" spans="1:11" x14ac:dyDescent="0.25">
@@ -13362,7 +13362,7 @@
         <v>67</v>
       </c>
       <c r="K291">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="292" spans="1:11" x14ac:dyDescent="0.25">
@@ -13397,7 +13397,7 @@
         <v>67</v>
       </c>
       <c r="K292">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="293" spans="1:11" x14ac:dyDescent="0.25">
@@ -13432,7 +13432,7 @@
         <v>67</v>
       </c>
       <c r="K293">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="294" spans="1:11" x14ac:dyDescent="0.25">
@@ -13467,7 +13467,7 @@
         <v>67</v>
       </c>
       <c r="K294">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="295" spans="1:11" x14ac:dyDescent="0.25">
@@ -13502,7 +13502,7 @@
         <v>67</v>
       </c>
       <c r="K295">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="296" spans="1:11" x14ac:dyDescent="0.25">
@@ -13537,7 +13537,7 @@
         <v>67</v>
       </c>
       <c r="K296">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.25">
@@ -13572,7 +13572,7 @@
         <v>67</v>
       </c>
       <c r="K297">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="298" spans="1:11" x14ac:dyDescent="0.25">
@@ -13607,7 +13607,7 @@
         <v>67</v>
       </c>
       <c r="K298">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="299" spans="1:11" x14ac:dyDescent="0.25">
@@ -13677,7 +13677,7 @@
         <v>67</v>
       </c>
       <c r="K300">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="301" spans="1:11" x14ac:dyDescent="0.25">
@@ -13712,7 +13712,7 @@
         <v>67</v>
       </c>
       <c r="K301">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>